<commit_message>
fix: 計算欄補 calculatedColumnFormula 根治 #REF! 地雷
問題：同仁 key 資料後多分頁不計算。
根因：Excel Table 的計算欄 cell 用 [@欄名] 結構引用，但 table XML
      缺少 calculatedColumnFormula 宣告。使用者一編輯/刪列，Excel
      就把 [@欄名] 崩成 #REF!，導致 案類分類 = #REF!，所有統計頁
      COUNTIFS(Tbl[案類分類],...) 全抓 0。

修法：
- phase2_data_tables.py：Tbl案件 6 計算欄補 calculatedColumnFormula
  （是否破獲/歸屬年度/案類分類/是否納入統計/主排序鍵/計入發生數）
- phase3_page8_drug.py：Tbl毒調 4 計算欄補
  （距今天數/是否到驗/狀態燈/候選旗標）
- 驗證 openpyxl load/save 與 phase 11 後仍保留宣告
- 全測試 1426/1426 維持綠燈
</commit_message>
<xml_diff>
--- a/build/output/PoliceStation_v2.0.xlsx
+++ b/build/output/PoliceStation_v2.0.xlsx
@@ -1835,7 +1835,6 @@
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Tbl案件" displayName="Tbl案件" ref="A14:Y218" headerRowCount="1">
-  <autoFilter ref="A14:Y218"/>
   <tableColumns count="25">
     <tableColumn id="1" name="編號"/>
     <tableColumn id="2" name="案類"/>
@@ -1854,13 +1853,25 @@
     <tableColumn id="15" name="涉案金額"/>
     <tableColumn id="16" name="建立日期"/>
     <tableColumn id="17" name="建立者"/>
-    <tableColumn id="18" name="是否破獲"/>
-    <tableColumn id="19" name="歸屬年度"/>
-    <tableColumn id="20" name="案類分類"/>
-    <tableColumn id="21" name="是否納入統計"/>
-    <tableColumn id="22" name="主排序鍵"/>
+    <tableColumn id="18" name="是否破獲">
+      <calculatedColumnFormula>IFERROR(IF(OR([@案件狀況]="已破獲未移送",[@案件狀況]="已移送"),"是","否"),"")</calculatedColumnFormula>
+    </tableColumn>
+    <tableColumn id="19" name="歸屬年度">
+      <calculatedColumnFormula>IFERROR(IF([@發生時間]="","",YEAR([@發生時間])-1911),"")</calculatedColumnFormula>
+    </tableColumn>
+    <tableColumn id="20" name="案類分類">
+      <calculatedColumnFormula>IFERROR(INDEX(案類分類清單,MATCH([@案類],案類名稱清單,0)),"")</calculatedColumnFormula>
+    </tableColumn>
+    <tableColumn id="21" name="是否納入統計">
+      <calculatedColumnFormula>IFERROR(INDEX(納入全般清單,MATCH([@案類],案類名稱清單,0)),"否")</calculatedColumnFormula>
+    </tableColumn>
+    <tableColumn id="22" name="主排序鍵">
+      <calculatedColumnFormula>IFERROR([@歸屬年度]*10000+IFERROR(MATCH([@案件狀況],{"尚未偵破","已破獲未移送","已移送","簽結"},0),0)*100+ROW(),0)</calculatedColumnFormula>
+    </tableColumn>
     <tableColumn id="23" name="績效類別"/>
-    <tableColumn id="24" name="計入發生數"/>
+    <tableColumn id="24" name="計入發生數">
+      <calculatedColumnFormula>IFERROR(IF([@績效類別]="","是","否"),"是")</calculatedColumnFormula>
+    </tableColumn>
     <tableColumn id="25" name="自填案類"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -1869,7 +1880,6 @@
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="Tbl毒調" displayName="Tbl毒調" ref="A14:N84" headerRowCount="1">
-  <autoFilter ref="A14:N84"/>
   <tableColumns count="14">
     <tableColumn id="1" name="編號"/>
     <tableColumn id="2" name="姓名"/>
@@ -1881,10 +1891,18 @@
     <tableColumn id="8" name="管制情形"/>
     <tableColumn id="9" name="備註"/>
     <tableColumn id="10" name="最後到驗日"/>
-    <tableColumn id="11" name="距今天數"/>
-    <tableColumn id="12" name="是否到驗"/>
-    <tableColumn id="13" name="狀態燈"/>
-    <tableColumn id="14" name="候選旗標"/>
+    <tableColumn id="11" name="距今天數">
+      <calculatedColumnFormula>IFERROR(IF([@最後到驗日]="","",今日-[@最後到驗日]),"")</calculatedColumnFormula>
+    </tableColumn>
+    <tableColumn id="12" name="是否到驗">
+      <calculatedColumnFormula>IFERROR(IF([@管制情形]="",0,IF(OR(SUMPRODUCT(--ISNUMBER(SEARCH({"已驗","已到驗","通緝","強採","在監"},[@管制情形])))&gt;0,AND(ISNUMBER([@距今天數]),[@距今天數]&lt;=30)),1,0)),0)</calculatedColumnFormula>
+    </tableColumn>
+    <tableColumn id="13" name="狀態燈">
+      <calculatedColumnFormula>IFERROR(IF([@管制情形]="","○ 未填",IF(ISNUMBER(SEARCH("解除",[@管制情形])),"○ 結束",IF(AND(ISNUMBER([@距今天數]),[@距今天數]&gt;30),"● 紅",IF([@是否到驗]=1,"● 綠","⚠ 黃")))),"")</calculatedColumnFormula>
+    </tableColumn>
+    <tableColumn id="14" name="候選旗標">
+      <calculatedColumnFormula>IFERROR(IF(OR(ISNUMBER(SEARCH("未到驗",[@管制情形])),AND(ISNUMBER([@距今天數]),[@距今天數]&gt;30)),1,0),0)</calculatedColumnFormula>
+    </tableColumn>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium5" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1892,7 +1910,6 @@
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Tbl交通" displayName="Tbl交通" ref="A14:F119" headerRowCount="1">
-  <autoFilter ref="A14:F119"/>
   <tableColumns count="6">
     <tableColumn id="1" name="編號"/>
     <tableColumn id="2" name="取締日期"/>
@@ -1907,7 +1924,6 @@
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="Tbl歷史" displayName="Tbl歷史" ref="A10:N45" headerRowCount="1">
-  <autoFilter ref="A10:N45"/>
   <tableColumns count="14">
     <tableColumn id="1" name="統計年月"/>
     <tableColumn id="2" name="全般發生"/>

</xml_diff>